<commit_message>
feat(reports): accept the latest DSM statement format
</commit_message>
<xml_diff>
--- a/services/processing/app/v2/exchange_reports/samples/DSM Report Sample.xlsx
+++ b/services/processing/app/v2/exchange_reports/samples/DSM Report Sample.xlsx
@@ -1,40 +1,84 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="6030"/>
   </bookViews>
   <sheets>
-    <sheet name="DSM Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="DSM Report" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Schedule Total</t>
+  </si>
+  <si>
+    <t>Actual Total</t>
+  </si>
+  <si>
+    <t>Frequency</t>
+  </si>
+  <si>
+    <t>Deviation Rate</t>
+  </si>
+  <si>
+    <t>Deviation</t>
+  </si>
+  <si>
+    <t>Overdrawl_Charges</t>
+  </si>
+  <si>
+    <t>Underdrawl_Charges</t>
+  </si>
+  <si>
+    <t>Postfacto_Charges</t>
+  </si>
+  <si>
+    <t>dev_%</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="DD-MM-YYYY"/>
-    <numFmt numFmtId="165" formatCode="HH:MM"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -52,87 +96,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,127 +403,114 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="8" width="11" customWidth="1"/>
+    <col min="9" max="9" width="19" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Time</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Schedule Total</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Actual Total</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Frequency</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Deviation Rate</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Deviation</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Overdrawl_Charges</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Underdrawl_Charges</t>
-        </is>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="5" t="n">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
         <v>45658</v>
       </c>
-      <c r="B2" s="6" t="n">
+      <c r="B2" s="4">
         <v>0</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="2">
         <v>100</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="2">
         <v>98.5</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="2">
         <v>50.01</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="F2" s="2">
         <v>450</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G2" s="2">
         <v>-1.5</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="H2" s="2"/>
+      <c r="I2" s="2">
         <v>0</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="J2" s="2">
         <v>1687.5</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="5" t="n">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
         <v>45658</v>
       </c>
-      <c r="B3" s="6" t="n">
-        <v>0.01041666666666667</v>
-      </c>
-      <c r="C3" s="4" t="n">
+      <c r="B3" s="4">
+        <v>1.041666666666667E-2</v>
+      </c>
+      <c r="C3" s="2">
         <v>100</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="2">
         <v>101.2</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="2">
         <v>49.98</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="2">
         <v>520</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="2">
         <v>1.2</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H3" s="2"/>
+      <c r="I3" s="2">
         <v>1560</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="J3" s="2">
         <v>0</v>
       </c>
     </row>

</xml_diff>